<commit_message>
nueva base y nuevo lotes
</commit_message>
<xml_diff>
--- a/LABORES AGRICOLAS/LOTESH.xlsx
+++ b/LABORES AGRICOLAS/LOTESH.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PEDRO\Produccion-Lamiformi\cv-20250714T161904Z-1-001\cv\2025\SISBANLAM2025\Merejildo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1912DFEE-047A-4A91-BDB0-D1F14E463742}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C73E0372-C7AF-46E2-9B75-F0472FBEEA2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="10">
   <si>
     <t>SECTOR</t>
   </si>
@@ -34,9 +34,6 @@
     <t>JEFE</t>
   </si>
   <si>
-    <t>AN</t>
-  </si>
-  <si>
     <t>FREDDY SUAREZ</t>
   </si>
   <si>
@@ -47,6 +44,12 @@
   </si>
   <si>
     <t>LUIS DOMINGUEZ</t>
+  </si>
+  <si>
+    <t>HACIENDA</t>
+  </si>
+  <si>
+    <t>SAN HUMBERTO</t>
   </si>
 </sst>
 </file>
@@ -126,7 +129,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -244,15 +247,6 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
       <right style="thin">
         <color indexed="64"/>
       </right>
@@ -268,7 +262,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -315,11 +309,8 @@
     <xf numFmtId="0" fontId="3" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="2" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="164" fontId="1" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -602,13 +593,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D28"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="20.140625" customWidth="1"/>
+    <col min="5" max="5" width="16.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -618,11 +610,14 @@
       <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="18" t="s">
+      <c r="D1" s="17" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="E1" s="17" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="4">
         <v>1</v>
       </c>
@@ -632,11 +627,14 @@
       <c r="C2" s="6">
         <v>10.34</v>
       </c>
-      <c r="D2" s="17" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="D2" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="4">
         <v>1</v>
       </c>
@@ -646,11 +644,14 @@
       <c r="C3" s="6">
         <v>10.039999999999999</v>
       </c>
-      <c r="D3" s="17" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="D3" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="E3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="4">
         <v>1</v>
       </c>
@@ -660,11 +661,14 @@
       <c r="C4" s="6">
         <v>10</v>
       </c>
-      <c r="D4" s="17" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="D4" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="E4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" s="4">
         <v>1</v>
       </c>
@@ -674,11 +678,14 @@
       <c r="C5" s="6">
         <v>10.130000000000001</v>
       </c>
-      <c r="D5" s="17" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="D5" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="E5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="4">
         <v>1</v>
       </c>
@@ -688,11 +695,14 @@
       <c r="C6" s="6">
         <v>10</v>
       </c>
-      <c r="D6" s="17" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="D6" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="E6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="4">
         <v>1</v>
       </c>
@@ -702,11 +712,14 @@
       <c r="C7" s="6">
         <v>10.130000000000001</v>
       </c>
-      <c r="D7" s="17" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="D7" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="E7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="4">
         <v>1</v>
       </c>
@@ -716,11 +729,14 @@
       <c r="C8" s="6">
         <v>10</v>
       </c>
-      <c r="D8" s="17" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="D8" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="E8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A9" s="7">
         <v>2</v>
       </c>
@@ -730,11 +746,14 @@
       <c r="C9" s="8">
         <v>10</v>
       </c>
-      <c r="D9" s="17" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="D9" s="16" t="s">
+        <v>5</v>
+      </c>
+      <c r="E9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
         <v>2</v>
       </c>
@@ -744,11 +763,14 @@
       <c r="C10" s="8">
         <v>10</v>
       </c>
-      <c r="D10" s="17" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="D10" s="16" t="s">
+        <v>5</v>
+      </c>
+      <c r="E10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A11" s="7">
         <v>2</v>
       </c>
@@ -758,11 +780,14 @@
       <c r="C11" s="8">
         <v>10.01</v>
       </c>
-      <c r="D11" s="17" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="D11" s="16" t="s">
+        <v>5</v>
+      </c>
+      <c r="E11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A12" s="7">
         <v>2</v>
       </c>
@@ -772,11 +797,14 @@
       <c r="C12" s="8">
         <v>10.08</v>
       </c>
-      <c r="D12" s="17" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="D12" s="16" t="s">
+        <v>5</v>
+      </c>
+      <c r="E12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A13" s="7">
         <v>2</v>
       </c>
@@ -786,11 +814,14 @@
       <c r="C13" s="8">
         <v>10</v>
       </c>
-      <c r="D13" s="17" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="D13" s="16" t="s">
+        <v>5</v>
+      </c>
+      <c r="E13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A14" s="7">
         <v>2</v>
       </c>
@@ -800,11 +831,14 @@
       <c r="C14" s="8">
         <v>10</v>
       </c>
-      <c r="D14" s="17" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="D14" s="16" t="s">
+        <v>5</v>
+      </c>
+      <c r="E14" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A15" s="7">
         <v>2</v>
       </c>
@@ -814,11 +848,14 @@
       <c r="C15" s="8">
         <v>10.01</v>
       </c>
-      <c r="D15" s="17" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="D15" s="16" t="s">
+        <v>5</v>
+      </c>
+      <c r="E15" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A16" s="9">
         <v>3</v>
       </c>
@@ -828,11 +865,14 @@
       <c r="C16" s="10">
         <v>10.11</v>
       </c>
-      <c r="D16" s="17" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="D16" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="E16" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A17" s="9">
         <v>3</v>
       </c>
@@ -842,11 +882,14 @@
       <c r="C17" s="10">
         <v>10</v>
       </c>
-      <c r="D17" s="17" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="D17" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="E17" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A18" s="7">
         <v>2</v>
       </c>
@@ -856,11 +899,14 @@
       <c r="C18" s="8">
         <v>10</v>
       </c>
-      <c r="D18" s="17" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="D18" s="16" t="s">
+        <v>5</v>
+      </c>
+      <c r="E18" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A19" s="9">
         <v>3</v>
       </c>
@@ -870,11 +916,14 @@
       <c r="C19" s="12">
         <v>10.25</v>
       </c>
-      <c r="D19" s="17" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="D19" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="E19" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A20" s="9">
         <v>3</v>
       </c>
@@ -884,11 +933,14 @@
       <c r="C20" s="12">
         <v>10</v>
       </c>
-      <c r="D20" s="17" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="D20" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="E20" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A21" s="9">
         <v>3</v>
       </c>
@@ -898,11 +950,14 @@
       <c r="C21" s="12">
         <v>10.31</v>
       </c>
-      <c r="D21" s="17" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="D21" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="E21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A22" s="9">
         <v>3</v>
       </c>
@@ -912,11 +967,14 @@
       <c r="C22" s="12">
         <v>10</v>
       </c>
-      <c r="D22" s="17" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="D22" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="E22" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A23" s="9">
         <v>3</v>
       </c>
@@ -926,11 +984,14 @@
       <c r="C23" s="12">
         <v>10</v>
       </c>
-      <c r="D23" s="17" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="D23" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="E23" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A24" s="13">
         <v>4</v>
       </c>
@@ -940,11 +1001,14 @@
       <c r="C24" s="14">
         <v>10.5</v>
       </c>
-      <c r="D24" s="17" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="D24" s="16" t="s">
+        <v>7</v>
+      </c>
+      <c r="E24" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A25" s="13">
         <v>4</v>
       </c>
@@ -954,11 +1018,14 @@
       <c r="C25" s="14">
         <v>10.5</v>
       </c>
-      <c r="D25" s="17" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="D25" s="16" t="s">
+        <v>7</v>
+      </c>
+      <c r="E25" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A26" s="13">
         <v>4</v>
       </c>
@@ -968,11 +1035,14 @@
       <c r="C26" s="14">
         <v>10.5</v>
       </c>
-      <c r="D26" s="17" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D26" s="16" t="s">
+        <v>7</v>
+      </c>
+      <c r="E26" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="15">
         <v>4</v>
       </c>
@@ -982,22 +1052,113 @@
       <c r="C27" s="14">
         <v>10</v>
       </c>
-      <c r="D27" s="17" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="15" t="s">
-        <v>4</v>
-      </c>
-      <c r="B28" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="C28" s="16">
-        <v>40</v>
-      </c>
-      <c r="D28" s="17" t="s">
-        <v>8</v>
+      <c r="D27" s="16" t="s">
+        <v>7</v>
+      </c>
+      <c r="E27" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="15">
+        <v>4</v>
+      </c>
+      <c r="B28" s="5">
+        <v>27</v>
+      </c>
+      <c r="C28" s="14">
+        <v>10</v>
+      </c>
+      <c r="D28" s="16" t="s">
+        <v>7</v>
+      </c>
+      <c r="E28" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="15">
+        <v>4</v>
+      </c>
+      <c r="B29" s="5">
+        <v>28</v>
+      </c>
+      <c r="C29" s="14">
+        <v>10</v>
+      </c>
+      <c r="D29" s="16" t="s">
+        <v>7</v>
+      </c>
+      <c r="E29" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="15">
+        <v>4</v>
+      </c>
+      <c r="B30" s="5">
+        <v>29</v>
+      </c>
+      <c r="C30" s="14">
+        <v>10</v>
+      </c>
+      <c r="D30" s="16" t="s">
+        <v>7</v>
+      </c>
+      <c r="E30" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="15">
+        <v>4</v>
+      </c>
+      <c r="B31" s="5">
+        <v>30</v>
+      </c>
+      <c r="C31" s="14">
+        <v>10</v>
+      </c>
+      <c r="D31" s="16" t="s">
+        <v>7</v>
+      </c>
+      <c r="E31" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="15">
+        <v>4</v>
+      </c>
+      <c r="B32" s="5">
+        <v>31</v>
+      </c>
+      <c r="C32" s="14">
+        <v>10</v>
+      </c>
+      <c r="D32" s="16" t="s">
+        <v>7</v>
+      </c>
+      <c r="E32" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="15">
+        <v>4</v>
+      </c>
+      <c r="B33" s="5">
+        <v>32</v>
+      </c>
+      <c r="C33" s="14">
+        <v>10</v>
+      </c>
+      <c r="D33" s="16" t="s">
+        <v>7</v>
+      </c>
+      <c r="E33" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>